<commit_message>
WiP on solutes in runoff
</commit_message>
<xml_diff>
--- a/Examples/Tutorials/SoluteInRunoffCalcs.xlsx
+++ b/Examples/Tutorials/SoluteInRunoffCalcs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\aaUnderVC\ApsimX\Examples\Tutorials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED61B36-2CB0-4944-96B9-2EFF515EC6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D89FDB-2B9F-4A40-99DF-A0B914807A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22650" yWindow="975" windowWidth="24495" windowHeight="19635" xr2:uid="{457C1435-C66A-40C7-B0EF-CBB12B028E2E}"/>
   </bookViews>
@@ -107,9 +107,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1701,7 +1700,7 @@
         <v>5</v>
       </c>
       <c r="B13">
-        <f>IF(A13&lt;=$A$2,($A$2/A13)^2,0)</f>
+        <f t="shared" ref="B13:B18" si="0">IF(A13&lt;=$A$2,($A$2/A13)^2,0)</f>
         <v>36</v>
       </c>
       <c r="F13">
@@ -1710,8 +1709,8 @@
       <c r="G13">
         <v>1</v>
       </c>
-      <c r="H13" s="1">
-        <f>MIN(1,MAX(0,1-(G13-$G$1)/($G$2-$G$1)))</f>
+      <c r="H13">
+        <f t="shared" ref="H13:H34" si="1">MIN(1,MAX(0,1-(G13-$G$1)/($G$2-$G$1)))</f>
         <v>1</v>
       </c>
       <c r="I13">
@@ -1728,7 +1727,7 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <f>IF(A14&lt;=$A$2,($A$2/A14)^2,0)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="F14">
@@ -1737,16 +1736,16 @@
       <c r="G14">
         <v>3</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14">
         <f>MIN(1,MAX(0,1-(G14-$G$1)/($G$2-$G$1)))</f>
         <v>1</v>
       </c>
       <c r="I14">
-        <f t="shared" ref="I14:I34" si="0">MIN(1,$G$9/$G$4)</f>
+        <f t="shared" ref="I14:I34" si="2">MIN(1,$G$9/$G$4)</f>
         <v>1</v>
       </c>
       <c r="J14">
-        <f t="shared" ref="J14:J34" si="1">H14*I14*$G$5*F14</f>
+        <f t="shared" ref="J14:J34" si="3">H14*I14*$G$5*F14</f>
         <v>22.5</v>
       </c>
     </row>
@@ -1755,7 +1754,7 @@
         <v>25</v>
       </c>
       <c r="B15">
-        <f>IF(A15&lt;=$A$2,($A$2/A15)^2,0)</f>
+        <f t="shared" si="0"/>
         <v>1.44</v>
       </c>
       <c r="F15">
@@ -1764,16 +1763,16 @@
       <c r="G15">
         <v>5</v>
       </c>
-      <c r="H15" s="1">
-        <f>MIN(1,MAX(0,1-(G15-$G$1)/($G$2-$G$1)))</f>
+      <c r="H15">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>22.5</v>
       </c>
     </row>
@@ -1782,7 +1781,7 @@
         <v>35</v>
       </c>
       <c r="B16">
-        <f>IF(A16&lt;=$A$2,($A$2/A16)^2,0)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F16">
@@ -1791,16 +1790,16 @@
       <c r="G16">
         <v>7</v>
       </c>
-      <c r="H16" s="1">
-        <f>MIN(1,MAX(0,1-(G16-$G$1)/($G$2-$G$1)))</f>
+      <c r="H16">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>22.5</v>
       </c>
     </row>
@@ -1809,7 +1808,7 @@
         <v>45</v>
       </c>
       <c r="B17">
-        <f>IF(A17&lt;=$A$2,($A$2/A17)^2,0)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F17">
@@ -1818,16 +1817,16 @@
       <c r="G17">
         <v>9</v>
       </c>
-      <c r="H17" s="1">
-        <f>MIN(1,MAX(0,1-(G17-$G$1)/($G$2-$G$1)))</f>
+      <c r="H17">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>22.5</v>
       </c>
     </row>
@@ -1836,7 +1835,7 @@
         <v>55</v>
       </c>
       <c r="B18">
-        <f>IF(A18&lt;=$A$2,($A$2/A18)^2,0)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F18">
@@ -1845,16 +1844,16 @@
       <c r="G18">
         <v>11</v>
       </c>
-      <c r="H18" s="1">
-        <f>MIN(1,MAX(0,1-(G18-$G$1)/($G$2-$G$1)))</f>
+      <c r="H18">
+        <f t="shared" si="1"/>
         <v>0.95</v>
       </c>
       <c r="I18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>21.375</v>
       </c>
     </row>
@@ -1865,16 +1864,16 @@
       <c r="G19">
         <v>13</v>
       </c>
-      <c r="H19" s="1">
-        <f>MIN(1,MAX(0,1-(G19-$G$1)/($G$2-$G$1)))</f>
+      <c r="H19">
+        <f t="shared" si="1"/>
         <v>0.85</v>
       </c>
       <c r="I19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>19.125</v>
       </c>
     </row>
@@ -1885,16 +1884,16 @@
       <c r="G20">
         <v>15</v>
       </c>
-      <c r="H20" s="1">
-        <f>MIN(1,MAX(0,1-(G20-$G$1)/($G$2-$G$1)))</f>
+      <c r="H20">
+        <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
       <c r="I20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>16.875</v>
       </c>
     </row>
@@ -1903,7 +1902,7 @@
         <v>1</v>
       </c>
       <c r="B21">
-        <f>IF(A21&lt;=$A$2,($A$2/A21)^2,0)</f>
+        <f t="shared" ref="B21:B30" si="4">IF(A21&lt;=$A$2,($A$2/A21)^2,0)</f>
         <v>900</v>
       </c>
       <c r="F21">
@@ -1912,16 +1911,16 @@
       <c r="G21">
         <v>17</v>
       </c>
-      <c r="H21" s="1">
-        <f>MIN(1,MAX(0,1-(G21-$G$1)/($G$2-$G$1)))</f>
+      <c r="H21">
+        <f t="shared" si="1"/>
         <v>0.65</v>
       </c>
       <c r="I21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>14.625000000000002</v>
       </c>
     </row>
@@ -1930,7 +1929,7 @@
         <v>2</v>
       </c>
       <c r="B22">
-        <f>IF(A22&lt;=$A$2,($A$2/A22)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>225</v>
       </c>
       <c r="F22">
@@ -1939,16 +1938,16 @@
       <c r="G22">
         <v>19</v>
       </c>
-      <c r="H22" s="1">
-        <f>MIN(1,MAX(0,1-(G22-$G$1)/($G$2-$G$1)))</f>
+      <c r="H22">
+        <f t="shared" si="1"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="I22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12.375000000000002</v>
       </c>
     </row>
@@ -1957,7 +1956,7 @@
         <v>3</v>
       </c>
       <c r="B23">
-        <f>IF(A23&lt;=$A$2,($A$2/A23)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>100</v>
       </c>
       <c r="F23">
@@ -1966,16 +1965,16 @@
       <c r="G23">
         <v>21</v>
       </c>
-      <c r="H23" s="1">
-        <f>MIN(1,MAX(0,1-(G23-$G$1)/($G$2-$G$1)))</f>
+      <c r="H23">
+        <f t="shared" si="1"/>
         <v>0.44999999999999996</v>
       </c>
       <c r="I23">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>10.125</v>
       </c>
     </row>
@@ -1984,7 +1983,7 @@
         <v>4</v>
       </c>
       <c r="B24">
-        <f>IF(A24&lt;=$A$2,($A$2/A24)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>56.25</v>
       </c>
       <c r="F24">
@@ -1993,16 +1992,16 @@
       <c r="G24">
         <v>23</v>
       </c>
-      <c r="H24" s="1">
-        <f>MIN(1,MAX(0,1-(G24-$G$1)/($G$2-$G$1)))</f>
+      <c r="H24">
+        <f t="shared" si="1"/>
         <v>0.35</v>
       </c>
       <c r="I24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7.875</v>
       </c>
     </row>
@@ -2011,7 +2010,7 @@
         <v>5</v>
       </c>
       <c r="B25">
-        <f>IF(A25&lt;=$A$2,($A$2/A25)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>36</v>
       </c>
       <c r="F25">
@@ -2020,16 +2019,16 @@
       <c r="G25">
         <v>25</v>
       </c>
-      <c r="H25" s="1">
-        <f>MIN(1,MAX(0,1-(G25-$G$1)/($G$2-$G$1)))</f>
+      <c r="H25">
+        <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
       <c r="I25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.625</v>
       </c>
     </row>
@@ -2038,7 +2037,7 @@
         <v>6</v>
       </c>
       <c r="B26">
-        <f>IF(A26&lt;=$A$2,($A$2/A26)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>25</v>
       </c>
       <c r="F26">
@@ -2047,16 +2046,16 @@
       <c r="G26">
         <v>27</v>
       </c>
-      <c r="H26" s="1">
-        <f>MIN(1,MAX(0,1-(G26-$G$1)/($G$2-$G$1)))</f>
+      <c r="H26">
+        <f t="shared" si="1"/>
         <v>0.15000000000000002</v>
       </c>
       <c r="I26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>3.3750000000000009</v>
       </c>
     </row>
@@ -2065,7 +2064,7 @@
         <v>7</v>
       </c>
       <c r="B27">
-        <f>IF(A27&lt;=$A$2,($A$2/A27)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>18.367346938775508</v>
       </c>
       <c r="F27">
@@ -2074,16 +2073,16 @@
       <c r="G27">
         <v>29</v>
       </c>
-      <c r="H27" s="1">
-        <f>MIN(1,MAX(0,1-(G27-$G$1)/($G$2-$G$1)))</f>
+      <c r="H27">
+        <f t="shared" si="1"/>
         <v>5.0000000000000044E-2</v>
       </c>
       <c r="I27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>1.1250000000000009</v>
       </c>
     </row>
@@ -2092,7 +2091,7 @@
         <v>8</v>
       </c>
       <c r="B28">
-        <f>IF(A28&lt;=$A$2,($A$2/A28)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>14.0625</v>
       </c>
       <c r="F28">
@@ -2101,16 +2100,16 @@
       <c r="G28">
         <v>31</v>
       </c>
-      <c r="H28" s="1">
-        <f>MIN(1,MAX(0,1-(G28-$G$1)/($G$2-$G$1)))</f>
+      <c r="H28">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I28">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2119,7 +2118,7 @@
         <v>9</v>
       </c>
       <c r="B29">
-        <f>IF(A29&lt;=$A$2,($A$2/A29)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>11.111111111111112</v>
       </c>
       <c r="F29">
@@ -2128,16 +2127,16 @@
       <c r="G29">
         <v>33</v>
       </c>
-      <c r="H29" s="1">
-        <f>MIN(1,MAX(0,1-(G29-$G$1)/($G$2-$G$1)))</f>
+      <c r="H29">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I29">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2146,7 +2145,7 @@
         <v>10</v>
       </c>
       <c r="B30">
-        <f>IF(A30&lt;=$A$2,($A$2/A30)^2,0)</f>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="F30">
@@ -2155,18 +2154,18 @@
       <c r="G30">
         <v>35</v>
       </c>
-      <c r="H30" s="1">
-        <f>MIN(1,MAX(0,1-(G30-$G$1)/($G$2-$G$1)))</f>
-        <v>0</v>
-      </c>
-      <c r="I30">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J30">
+      <c r="H30">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I30">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F31">
@@ -2175,18 +2174,18 @@
       <c r="G31">
         <v>37</v>
       </c>
-      <c r="H31" s="1">
-        <f>MIN(1,MAX(0,1-(G31-$G$1)/($G$2-$G$1)))</f>
-        <v>0</v>
-      </c>
-      <c r="I31">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J31">
+      <c r="H31">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I31">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F32">
@@ -2195,18 +2194,18 @@
       <c r="G32">
         <v>39</v>
       </c>
-      <c r="H32" s="1">
-        <f>MIN(1,MAX(0,1-(G32-$G$1)/($G$2-$G$1)))</f>
-        <v>0</v>
-      </c>
-      <c r="I32">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J32">
+      <c r="H32">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I32">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F33">
@@ -2215,18 +2214,18 @@
       <c r="G33">
         <v>41</v>
       </c>
-      <c r="H33" s="1">
-        <f>MIN(1,MAX(0,1-(G33-$G$1)/($G$2-$G$1)))</f>
-        <v>0</v>
-      </c>
-      <c r="I33">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J33">
+      <c r="H33">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I33">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F34">
@@ -2235,16 +2234,16 @@
       <c r="G34">
         <v>43</v>
       </c>
-      <c r="H34" s="1">
-        <f>MIN(1,MAX(0,1-(G34-$G$1)/($G$2-$G$1)))</f>
+      <c r="H34">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>